<commit_message>
Configure date formatting and prepare for public deployment
</commit_message>
<xml_diff>
--- a/Import-data/sales_data.xlsx
+++ b/Import-data/sales_data.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sales_Data" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -514,10 +514,8 @@
           <t>North America</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>1299.00</t>
-        </is>
+      <c r="G2" t="n">
+        <v>1299</v>
       </c>
       <c r="H2" t="n">
         <v>2</v>
@@ -579,10 +577,8 @@
           <t>Europe</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>45.99</t>
-        </is>
+      <c r="G3" t="n">
+        <v>45.99</v>
       </c>
       <c r="H3" t="n">
         <v>5</v>
@@ -621,7 +617,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>01/02/2025</t>
+          <t>02/01/2025</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -644,10 +640,8 @@
           <t>Asia Pacific</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>799.00</t>
-        </is>
+      <c r="G4" t="n">
+        <v>799</v>
       </c>
       <c r="H4" t="n">
         <v>1</v>
@@ -686,7 +680,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>01/02/2025</t>
+          <t>02/01/2025</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -709,10 +703,8 @@
           <t>North America</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>349.00</t>
-        </is>
+      <c r="G5" t="n">
+        <v>349</v>
       </c>
       <c r="H5" t="n">
         <v>3</v>
@@ -751,7 +743,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>01/03/2025</t>
+          <t>03/01/2025</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -774,10 +766,8 @@
           <t>Europe</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>89.99</t>
-        </is>
+      <c r="G6" t="n">
+        <v>89.98999999999999</v>
       </c>
       <c r="H6" t="n">
         <v>10</v>
@@ -816,7 +806,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>01/03/2025</t>
+          <t>03/01/2025</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -839,10 +829,8 @@
           <t>Latin America</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>999.00</t>
-        </is>
+      <c r="G7" t="n">
+        <v>999</v>
       </c>
       <c r="H7" t="n">
         <v>1</v>
@@ -881,7 +869,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>01/04/2025</t>
+          <t>04/01/2025</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -904,10 +892,8 @@
           <t>Asia Pacific</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>79.99</t>
-        </is>
+      <c r="G8" t="n">
+        <v>79.98999999999999</v>
       </c>
       <c r="H8" t="n">
         <v>4</v>
@@ -946,7 +932,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>01/04/2025</t>
+          <t>04/01/2025</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -969,10 +955,8 @@
           <t>North America</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>129.99</t>
-        </is>
+      <c r="G9" t="n">
+        <v>129.99</v>
       </c>
       <c r="H9" t="n">
         <v>2</v>
@@ -1011,7 +995,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>01/05/2025</t>
+          <t>05/01/2025</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1034,10 +1018,8 @@
           <t>Europe</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>499.00</t>
-        </is>
+      <c r="G10" t="n">
+        <v>499</v>
       </c>
       <c r="H10" t="n">
         <v>3</v>
@@ -1076,7 +1058,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>01/05/2025</t>
+          <t>05/01/2025</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1099,10 +1081,8 @@
           <t>Asia Pacific</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>199.00</t>
-        </is>
+      <c r="G11" t="n">
+        <v>199</v>
       </c>
       <c r="H11" t="n">
         <v>5</v>
@@ -1141,7 +1121,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>01/06/2025</t>
+          <t>06/01/2025</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1164,10 +1144,8 @@
           <t>North America</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>1299.00</t>
-        </is>
+      <c r="G12" t="n">
+        <v>1299</v>
       </c>
       <c r="H12" t="n">
         <v>1</v>
@@ -1206,7 +1184,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>01/06/2025</t>
+          <t>06/01/2025</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1229,10 +1207,8 @@
           <t>Europe</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>45.99</t>
-        </is>
+      <c r="G13" t="n">
+        <v>45.99</v>
       </c>
       <c r="H13" t="n">
         <v>8</v>
@@ -1271,7 +1247,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>01/07/2025</t>
+          <t>07/01/2025</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1294,10 +1270,8 @@
           <t>Latin America</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>799.00</t>
-        </is>
+      <c r="G14" t="n">
+        <v>799</v>
       </c>
       <c r="H14" t="n">
         <v>2</v>
@@ -1336,7 +1310,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>01/07/2025</t>
+          <t>07/01/2025</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1359,10 +1333,8 @@
           <t>Asia Pacific</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>349.00</t>
-        </is>
+      <c r="G15" t="n">
+        <v>349</v>
       </c>
       <c r="H15" t="n">
         <v>6</v>
@@ -1401,7 +1373,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>01/08/2025</t>
+          <t>08/01/2025</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1424,10 +1396,8 @@
           <t>North America</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>89.99</t>
-        </is>
+      <c r="G16" t="n">
+        <v>89.98999999999999</v>
       </c>
       <c r="H16" t="n">
         <v>15</v>
@@ -1466,7 +1436,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>01/08/2025</t>
+          <t>08/01/2025</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1489,10 +1459,8 @@
           <t>Europe</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>999.00</t>
-        </is>
+      <c r="G17" t="n">
+        <v>999</v>
       </c>
       <c r="H17" t="n">
         <v>2</v>
@@ -1531,7 +1499,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>01/09/2025</t>
+          <t>09/01/2025</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1554,10 +1522,8 @@
           <t>North America</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>79.99</t>
-        </is>
+      <c r="G18" t="n">
+        <v>79.98999999999999</v>
       </c>
       <c r="H18" t="n">
         <v>8</v>
@@ -1596,7 +1562,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>01/09/2025</t>
+          <t>09/01/2025</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1619,10 +1585,8 @@
           <t>Asia Pacific</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>129.99</t>
-        </is>
+      <c r="G19" t="n">
+        <v>129.99</v>
       </c>
       <c r="H19" t="n">
         <v>3</v>
@@ -1661,7 +1625,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>01/10/2025</t>
+          <t>10/01/2025</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1684,10 +1648,8 @@
           <t>Latin America</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>499.00</t>
-        </is>
+      <c r="G20" t="n">
+        <v>499</v>
       </c>
       <c r="H20" t="n">
         <v>4</v>
@@ -1726,7 +1688,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>01/10/2025</t>
+          <t>10/01/2025</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1749,10 +1711,8 @@
           <t>Europe</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>199.00</t>
-        </is>
+      <c r="G21" t="n">
+        <v>199</v>
       </c>
       <c r="H21" t="n">
         <v>6</v>

</xml_diff>